<commit_message>
Complex changes but feels good progress
</commit_message>
<xml_diff>
--- a/Output/trading_journal_live.xlsx
+++ b/Output/trading_journal_live.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/261a4915364edc4c/Coding/Projects/Trading Journal/Output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_B0CB5FAC5D2E1657FE6579C669708EE57CBD87FD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B8A7AA4C-54C4-4DFD-A747-C2B61BB49BCA}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_EC015F8EDC37BE565AE434863412A5F656F9509E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{698E0D61-64C4-4665-8CF7-017DBD34CA5E}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Improvements" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1106" uniqueCount="429">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1126" uniqueCount="430">
   <si>
     <t>Sheet</t>
   </si>
@@ -322,6 +322,12 @@
     <t>Apr 19, 2024</t>
   </si>
   <si>
+    <t>Rich SPY</t>
+  </si>
+  <si>
+    <t>Fumbled</t>
+  </si>
+  <si>
     <t>OPTION</t>
   </si>
   <si>
@@ -331,6 +337,9 @@
     <t>Apr 15, 2024</t>
   </si>
   <si>
+    <t>Waited</t>
+  </si>
+  <si>
     <t>Feb 09, 2024</t>
   </si>
   <si>
@@ -679,12 +688,6 @@
     <t>11:33:36</t>
   </si>
   <si>
-    <t>Rich SPY</t>
-  </si>
-  <si>
-    <t>Fumbled</t>
-  </si>
-  <si>
     <t>3.45%</t>
   </si>
   <si>
@@ -1285,9 +1288,6 @@
     <t>Journal: 30D retro needs to be performed to determine if I was right or not. Probably can be automated based on Price.</t>
   </si>
   <si>
-    <t>Retro: Add due Retros</t>
-  </si>
-  <si>
     <t>Ideas: Taken ideas are missing a TradeID</t>
   </si>
   <si>
@@ -1334,16 +1334,20 @@
   </si>
   <si>
     <t>This log will keep track of all the trades we carry, including entry price, exit, tags and strategies which will be used for retrospectives. Based off Tradersyncs Export. Only fully executed trades will be included.</t>
+  </si>
+  <si>
+    <t>Retro: Perform due Retros</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="7" formatCode="&quot;$&quot;#,##0.00_);\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
   <fonts count="16" x14ac:knownFonts="1">
     <font>
@@ -1498,7 +1502,7 @@
     <xf numFmtId="9" fontId="8" fillId="0" borderId="1"/>
     <xf numFmtId="164" fontId="15" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1577,6 +1581,8 @@
     <xf numFmtId="14" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="7" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="currency" xfId="5" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
@@ -2544,160 +2550,160 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="G1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="H1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="I1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="J1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B3" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C3" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B4" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C4" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B7" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B8" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B9" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C9" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D9" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E9" s="31" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C10" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D10" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B11" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C11" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D11" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E11" s="31" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F11" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B12" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B13" t="s">
         <v>40</v>
@@ -2705,15 +2711,15 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B14" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B15" t="s">
         <v>40</v>
@@ -2721,7 +2727,7 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B16">
         <v>0.1</v>
@@ -2729,30 +2735,30 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B17" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C17" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B18" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C18" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D18" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E18" t="s">
         <v>60</v>
@@ -2761,124 +2767,124 @@
         <v>29</v>
       </c>
       <c r="G18" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B22" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B23" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C23" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B24" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B25" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B26" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B27" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B28" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B29" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B30" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C30" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B31" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B32" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B33" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B34" t="s">
         <v>40</v>
@@ -2886,7 +2892,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B35">
         <v>0.1</v>
@@ -2894,167 +2900,167 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B36" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C36" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D36" s="16" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B37" t="s">
-        <v>210</v>
+        <v>91</v>
       </c>
       <c r="C37" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D37" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B41" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C41" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D41" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B42" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C42" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B43" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C43" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B44" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B45" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B46" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B47" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C47" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D47" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E47" s="31" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B48" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C48" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D48" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B49" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C49" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D49" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E49" s="31" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F49" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B50" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C50" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B51" t="s">
         <v>40</v>
@@ -3062,15 +3068,15 @@
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B52" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B53" t="s">
         <v>40</v>
@@ -3078,7 +3084,7 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B54">
         <v>0.1</v>
@@ -3086,30 +3092,30 @@
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B55" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C55" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D55" s="16" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B56" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C56" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D56" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E56" t="s">
         <v>60</v>
@@ -3118,147 +3124,147 @@
         <v>29</v>
       </c>
       <c r="G56" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B60" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C60" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D60" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E60" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B61" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C61" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B62" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C62" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B63" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B64" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B65" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B66" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C66" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D66" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E66" s="31" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B67" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C67" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D67" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B68" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C68" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D68" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E68" s="31" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F68" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B69" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C69" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B70" t="s">
         <v>40</v>
@@ -3266,15 +3272,15 @@
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B71" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B72" t="s">
         <v>40</v>
@@ -3282,7 +3288,7 @@
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B73">
         <v>0.1</v>
@@ -3290,30 +3296,30 @@
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B74" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C74" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D74" s="16" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B75" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C75" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D75" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E75" t="s">
         <v>60</v>
@@ -3322,150 +3328,150 @@
         <v>29</v>
       </c>
       <c r="G75" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B79" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C79" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D79" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E79" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B80" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C80" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B81" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C81" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B82" s="31" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B83" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B84" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B85" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C85" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D85" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E85" s="31" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B86" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C86" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D86" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B87" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C87" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D87" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E87" s="31" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F87" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G87" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B88" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C88" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B89" t="s">
         <v>40</v>
@@ -3473,15 +3479,15 @@
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B90" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B91" t="s">
         <v>40</v>
@@ -3489,7 +3495,7 @@
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B92">
         <v>0.1</v>
@@ -3497,30 +3503,30 @@
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B93" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C93" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D93" s="16" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B94" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C94" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D94" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E94" t="s">
         <v>60</v>
@@ -3529,159 +3535,159 @@
         <v>29</v>
       </c>
       <c r="G94" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H94" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B98" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C98" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D98" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E98" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B99" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C99" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B100" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C100" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B101" s="31" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B102" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B103" s="31" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B104" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C104" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D104" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E104" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B105" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C105" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D105" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B106" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C106" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D106" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E106" s="31" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F106" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G106" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="H106" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B107" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C107" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D107" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B108" t="s">
         <v>40</v>
@@ -3689,15 +3695,15 @@
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B109" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B110" t="s">
         <v>40</v>
@@ -3705,7 +3711,7 @@
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B111">
         <v>0.1</v>
@@ -3713,30 +3719,30 @@
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B112" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C112" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D112" s="16" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B113" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C113" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D113" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E113" t="s">
         <v>60</v>
@@ -3745,165 +3751,165 @@
         <v>29</v>
       </c>
       <c r="G113" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H113" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B114" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B117" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C117" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D117" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E117" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B118" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C118" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B119" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C119" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B120" s="31" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B121" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B122" s="31" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C122" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B123" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C123" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D123" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E123" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B124" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C124" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D124" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B125" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C125" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D125" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E125" s="31" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F125" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="G125" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="H125" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I125" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B126" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C126" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B127" t="s">
         <v>40</v>
@@ -3911,15 +3917,15 @@
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B128" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="129" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B129" t="s">
         <v>40</v>
@@ -3927,7 +3933,7 @@
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B130">
         <v>0.1</v>
@@ -3935,188 +3941,188 @@
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B131" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C131" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D131" s="16" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B132" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C132" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D132" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E132" t="s">
         <v>60</v>
       </c>
       <c r="F132" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G132" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B133" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C133" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="135" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="136" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B136" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C136" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D136" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E136" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="137" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B137" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C137" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="138" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B138" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C138" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B139" s="31" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B140" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B141" s="31" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B142" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C142" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D142" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E142" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B143" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C143" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D143" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B144" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C144" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D144" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E144" s="31" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F144" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="G144" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="145" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B145" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C145" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="146" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B146" t="s">
         <v>40</v>
@@ -4124,15 +4130,15 @@
     </row>
     <row r="147" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B147" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B148" t="s">
         <v>40</v>
@@ -4140,7 +4146,7 @@
     </row>
     <row r="149" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B149">
         <v>0.1</v>
@@ -4148,150 +4154,150 @@
     </row>
     <row r="150" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B150" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C150" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D150" s="16" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="151" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B151" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C151" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D151" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E151" t="s">
         <v>60</v>
       </c>
       <c r="F151" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G151" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="152" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="154" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A154" s="1" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="155" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B155" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="156" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B156" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C156" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="157" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B157" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="158" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B158" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B159" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="160" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B160" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B161" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B162" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B164" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B165" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B166" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B167" t="s">
         <v>40</v>
@@ -4299,7 +4305,7 @@
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B168">
         <v>0.1</v>
@@ -4307,38 +4313,38 @@
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B169" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C169" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D169" s="16" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B170" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C170" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D170" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E170" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>
@@ -4359,42 +4365,42 @@
   <sheetData>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
@@ -4402,7 +4408,7 @@
         <v>2</v>
       </c>
       <c r="B13" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
@@ -4410,7 +4416,7 @@
         <v>3</v>
       </c>
       <c r="B14" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
@@ -4418,7 +4424,7 @@
         <v>29</v>
       </c>
       <c r="B15" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
@@ -4426,7 +4432,7 @@
         <v>30</v>
       </c>
       <c r="B16" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -4434,23 +4440,23 @@
         <v>31</v>
       </c>
       <c r="B17" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B18" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B19" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -4458,7 +4464,7 @@
         <v>5</v>
       </c>
       <c r="B20" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
@@ -4466,7 +4472,7 @@
         <v>6</v>
       </c>
       <c r="B21" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
@@ -4474,7 +4480,7 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
@@ -4482,7 +4488,7 @@
         <v>34</v>
       </c>
       <c r="B23" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
@@ -4490,12 +4496,12 @@
         <v>35</v>
       </c>
       <c r="B24" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
@@ -4503,7 +4509,7 @@
         <v>3</v>
       </c>
       <c r="B27" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.35">
@@ -4511,7 +4517,7 @@
         <v>2</v>
       </c>
       <c r="B28" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
@@ -4519,7 +4525,7 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.35">
@@ -4527,7 +4533,7 @@
         <v>45</v>
       </c>
       <c r="B30" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
@@ -4535,7 +4541,7 @@
         <v>46</v>
       </c>
       <c r="B31" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.35">
@@ -4543,7 +4549,7 @@
         <v>47</v>
       </c>
       <c r="B32" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
@@ -4551,7 +4557,7 @@
         <v>48</v>
       </c>
       <c r="B33" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
@@ -4559,7 +4565,7 @@
         <v>49</v>
       </c>
       <c r="B34" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.35">
@@ -4567,7 +4573,7 @@
         <v>50</v>
       </c>
       <c r="B35" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.35">
@@ -4575,7 +4581,7 @@
         <v>51</v>
       </c>
       <c r="B36" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
@@ -4583,7 +4589,7 @@
         <v>52</v>
       </c>
       <c r="B37" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
@@ -4591,7 +4597,7 @@
         <v>53</v>
       </c>
       <c r="B38" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.35">
@@ -4599,7 +4605,7 @@
         <v>54</v>
       </c>
       <c r="B39" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.35">
@@ -4607,7 +4613,7 @@
         <v>55</v>
       </c>
       <c r="B40" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.35">
@@ -4615,7 +4621,7 @@
         <v>56</v>
       </c>
       <c r="B41" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.35">
@@ -4623,7 +4629,7 @@
         <v>57</v>
       </c>
       <c r="B42" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.35">
@@ -4631,7 +4637,7 @@
         <v>58</v>
       </c>
       <c r="B43" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.35">
@@ -4639,19 +4645,19 @@
         <v>59</v>
       </c>
       <c r="B44" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C44" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D44" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E44" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="F44" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.35">
@@ -4659,7 +4665,7 @@
         <v>60</v>
       </c>
       <c r="B45" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.35">
@@ -4667,13 +4673,13 @@
         <v>61</v>
       </c>
       <c r="B46" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C46" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="D46" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.35">
@@ -4681,44 +4687,44 @@
         <v>62</v>
       </c>
       <c r="B47" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B50" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C50" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B51" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B52" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
@@ -4726,7 +4732,7 @@
         <v>62</v>
       </c>
       <c r="B55" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
@@ -4734,19 +4740,19 @@
         <v>59</v>
       </c>
       <c r="B56" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C56" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D56" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E56" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="F56" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.35">
@@ -4754,7 +4760,7 @@
         <v>84</v>
       </c>
       <c r="B57" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.35">
@@ -4762,7 +4768,7 @@
         <v>85</v>
       </c>
       <c r="B58" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
   </sheetData>
@@ -4781,37 +4787,37 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
@@ -4821,57 +4827,57 @@
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
   </sheetData>
@@ -4889,107 +4895,107 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>412</v>
+        <v>429</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
@@ -5052,7 +5058,7 @@
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
@@ -5082,7 +5088,7 @@
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
@@ -5092,7 +5098,7 @@
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
@@ -7838,10 +7844,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr codeName="Sheet4"/>
-  <dimension ref="A1:AA1"/>
+  <dimension ref="A1:AA5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="6" width="8.7265625" style="14" customWidth="1"/>
+    <col min="1" max="4" width="8.7265625" style="14" customWidth="1"/>
+    <col min="5" max="5" width="10.54296875" style="14" customWidth="1"/>
+    <col min="6" max="6" width="8.7265625" style="14" customWidth="1"/>
     <col min="7" max="7" width="18.08984375" style="14" customWidth="1"/>
     <col min="8" max="22" width="8.7265625" style="14" customWidth="1"/>
     <col min="23" max="23" width="14.81640625" style="12" customWidth="1"/>
@@ -7932,9 +7940,203 @@
         <v>87</v>
       </c>
     </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D2"/>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G2" s="36">
+        <v>45401</v>
+      </c>
+      <c r="H2" t="s">
+        <v>91</v>
+      </c>
+      <c r="N2" t="s">
+        <v>92</v>
+      </c>
+      <c r="S2" s="35">
+        <v>5.8</v>
+      </c>
+      <c r="T2" s="35">
+        <v>6</v>
+      </c>
+      <c r="U2" s="35">
+        <v>17.64</v>
+      </c>
+      <c r="V2" t="s">
+        <v>93</v>
+      </c>
+      <c r="W2" s="37">
+        <f>(T2-S2)/S2</f>
+        <v>3.4482758620689689E-2</v>
+      </c>
+      <c r="X2" s="35">
+        <v>-95</v>
+      </c>
+      <c r="Y2" s="35">
+        <v>20</v>
+      </c>
+      <c r="Z2" s="35"/>
+      <c r="AA2" s="37"/>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D3"/>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>95</v>
+      </c>
+      <c r="G3" s="36">
+        <v>45397</v>
+      </c>
+      <c r="S3" s="35">
+        <v>7.8</v>
+      </c>
+      <c r="T3" s="35">
+        <v>7.4</v>
+      </c>
+      <c r="U3" s="35">
+        <v>-42.36</v>
+      </c>
+      <c r="V3" t="s">
+        <v>93</v>
+      </c>
+      <c r="W3" s="37">
+        <f>(T3-S3)/S3</f>
+        <v>-5.1282051282051218E-2</v>
+      </c>
+      <c r="X3" s="35">
+        <v>-40</v>
+      </c>
+      <c r="Y3" s="35"/>
+      <c r="Z3" s="35"/>
+      <c r="AA3" s="37"/>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4"/>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4" t="s">
+        <v>95</v>
+      </c>
+      <c r="G4" s="36">
+        <v>45397</v>
+      </c>
+      <c r="H4" t="s">
+        <v>91</v>
+      </c>
+      <c r="I4" t="s">
+        <v>96</v>
+      </c>
+      <c r="S4" s="35">
+        <v>6.3</v>
+      </c>
+      <c r="T4" s="35">
+        <v>6.6</v>
+      </c>
+      <c r="U4" s="35">
+        <v>27.64</v>
+      </c>
+      <c r="V4" t="s">
+        <v>93</v>
+      </c>
+      <c r="W4" s="37">
+        <f>(T4-S4)/S4</f>
+        <v>4.7619047619047596E-2</v>
+      </c>
+      <c r="X4" s="35">
+        <v>20</v>
+      </c>
+      <c r="Y4" s="35">
+        <v>30</v>
+      </c>
+      <c r="Z4" s="35"/>
+      <c r="AA4" s="37"/>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5"/>
+      <c r="E5">
+        <v>25</v>
+      </c>
+      <c r="F5" t="s">
+        <v>97</v>
+      </c>
+      <c r="G5" s="36">
+        <v>45352</v>
+      </c>
+      <c r="S5" s="35">
+        <v>58.599899999999998</v>
+      </c>
+      <c r="T5" s="35">
+        <v>78.010000000000005</v>
+      </c>
+      <c r="U5" s="35">
+        <v>485.25</v>
+      </c>
+      <c r="V5" t="s">
+        <v>98</v>
+      </c>
+      <c r="W5" s="37">
+        <f>(T5-S5)/S5</f>
+        <v>0.33123094066713438</v>
+      </c>
+      <c r="X5" s="35">
+        <v>-58.247500000000002</v>
+      </c>
+      <c r="Y5" s="35">
+        <v>603.75300000000004</v>
+      </c>
+      <c r="Z5" s="35">
+        <v>674</v>
+      </c>
+      <c r="AA5" s="37">
+        <v>0.46010000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
@@ -7962,10 +8164,10 @@
         <v>67</v>
       </c>
       <c r="D1" s="17" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="F1" s="17" t="s">
         <v>79</v>
@@ -7983,7 +8185,7 @@
         <v>63</v>
       </c>
       <c r="K1" s="17" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="L1" s="17" t="s">
         <v>59</v>
@@ -7992,16 +8194,16 @@
         <v>60</v>
       </c>
       <c r="N1" s="17" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="O1" s="28" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="P1" s="25" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="Q1" s="25" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.35">
@@ -8019,7 +8221,7 @@
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
       <c r="N2" s="2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
@@ -9092,19 +9294,19 @@
         <v>50</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="E1" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="F1" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -9126,12 +9328,12 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B2" t="s">
         <v>36</v>
@@ -9156,34 +9358,34 @@
         <v>32</v>
       </c>
       <c r="B4" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C4" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="D4" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="E4" t="s">
         <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="G4" t="s">
         <v>41</v>
       </c>
       <c r="H4" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="I4" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="J4" t="s">
         <v>44</v>
       </c>
       <c r="K4" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="L4" t="s">
         <v>42</v>
@@ -9191,24 +9393,24 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B5" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C5" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D5" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E5" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
@@ -9216,22 +9418,22 @@
         <v>59</v>
       </c>
       <c r="B8" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C8" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E8" t="s">
+        <v>130</v>
+      </c>
+      <c r="F8" t="s">
+        <v>131</v>
+      </c>
+      <c r="G8" t="s">
         <v>126</v>
-      </c>
-      <c r="E8" t="s">
-        <v>127</v>
-      </c>
-      <c r="F8" t="s">
-        <v>128</v>
-      </c>
-      <c r="G8" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
@@ -9239,10 +9441,10 @@
         <v>49</v>
       </c>
       <c r="B9" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="C9" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
@@ -9250,34 +9452,34 @@
         <v>50</v>
       </c>
       <c r="B10" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C10" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="D10" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E10" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="F10" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="G10" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="H10" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="I10" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="J10" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="K10" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
@@ -9285,10 +9487,10 @@
         <v>54</v>
       </c>
       <c r="B11" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C11" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
@@ -9296,13 +9498,13 @@
         <v>60</v>
       </c>
       <c r="B12" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="C12" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D12" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
@@ -9310,18 +9512,18 @@
         <v>61</v>
       </c>
       <c r="B13" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C13" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="D13" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
@@ -9329,19 +9531,19 @@
         <v>59</v>
       </c>
       <c r="B16" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C16" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D16" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E16" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="F16" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -9378,28 +9580,28 @@
         <v>67</v>
       </c>
       <c r="F1" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="G1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="H1" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="I1" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J1" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="K1" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="L1" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="M1" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="N1" t="s">
         <v>79</v>
@@ -9411,64 +9613,64 @@
         <v>81</v>
       </c>
       <c r="Q1" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="R1" t="s">
         <v>58</v>
       </c>
       <c r="S1" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="T1" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="U1" t="s">
         <v>82</v>
       </c>
       <c r="V1" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="W1" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="X1" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="Y1" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="Z1" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="AA1" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="AB1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="AC1" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="AD1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="AE1" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="AF1" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="AG1" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="AH1" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="AI1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="AJ1" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="AK1" t="s">
         <v>84</v>
@@ -9477,10 +9679,10 @@
         <v>85</v>
       </c>
       <c r="AM1" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="AN1" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="AO1" t="s">
         <v>86</v>
@@ -9500,16 +9702,16 @@
         <v>25</v>
       </c>
       <c r="D2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="E2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="F2" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="G2" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="J2" s="35">
         <v>58.599899999999998</v>
@@ -9521,7 +9723,7 @@
         <v>485.25</v>
       </c>
       <c r="M2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="N2" s="35">
         <v>58.599899999999998</v>
@@ -9537,13 +9739,13 @@
         <v>0</v>
       </c>
       <c r="U2" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="V2" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="Y2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="Z2" s="35">
         <v>1465</v>
@@ -9553,16 +9755,16 @@
       </c>
       <c r="AB2" s="35"/>
       <c r="AD2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="AE2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="AF2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="AH2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="AI2" s="35">
         <v>19.41</v>
@@ -9585,25 +9787,25 @@
     </row>
     <row r="3" spans="1:42" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C3">
         <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="E3" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="F3" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="G3" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="J3" s="35">
         <v>175.91</v>
@@ -9622,13 +9824,13 @@
         <v>0</v>
       </c>
       <c r="U3" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="V3" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="Y3" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="Z3" s="35">
         <v>1583.19</v>
@@ -9638,19 +9840,19 @@
       </c>
       <c r="AB3" s="35"/>
       <c r="AD3" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="AE3" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="AF3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="AG3">
         <v>9</v>
       </c>
       <c r="AH3" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="AI3" s="35"/>
       <c r="AJ3">
@@ -9660,7 +9862,7 @@
     </row>
     <row r="4" spans="1:42" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B4" t="s">
         <v>27</v>
@@ -9669,16 +9871,16 @@
         <v>6</v>
       </c>
       <c r="D4" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="E4" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="F4" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="G4" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="J4" s="35">
         <v>170.19</v>
@@ -9697,13 +9899,13 @@
         <v>0</v>
       </c>
       <c r="U4" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="V4" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="Y4" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="Z4" s="35">
         <v>1021.14</v>
@@ -9713,19 +9915,19 @@
       </c>
       <c r="AB4" s="35"/>
       <c r="AD4" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="AE4" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="AF4" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="AG4">
         <v>6</v>
       </c>
       <c r="AH4" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="AI4" s="35"/>
       <c r="AJ4">
@@ -9735,25 +9937,25 @@
     </row>
     <row r="5" spans="1:42" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B5" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="C5">
         <v>75</v>
       </c>
       <c r="D5" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="E5" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F5" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="G5" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="J5" s="35">
         <v>26.55</v>
@@ -9772,13 +9974,13 @@
         <v>0</v>
       </c>
       <c r="U5" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="V5" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="Y5" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="Z5" s="35">
         <v>1990.5</v>
@@ -9788,19 +9990,19 @@
       </c>
       <c r="AB5" s="35"/>
       <c r="AD5" t="s">
+        <v>199</v>
+      </c>
+      <c r="AE5" t="s">
         <v>196</v>
       </c>
-      <c r="AE5" t="s">
-        <v>193</v>
-      </c>
       <c r="AF5" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="AG5">
         <v>75</v>
       </c>
       <c r="AH5" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="AI5" s="35"/>
       <c r="AJ5">
@@ -9810,7 +10012,7 @@
     </row>
     <row r="6" spans="1:42" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B6" t="s">
         <v>89</v>
@@ -9819,16 +10021,16 @@
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E6" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F6" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="G6" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="J6" s="35">
         <v>7.8</v>
@@ -9840,7 +10042,7 @@
         <v>-40</v>
       </c>
       <c r="M6" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="N6" s="35">
         <v>7.8</v>
@@ -9855,19 +10057,19 @@
         <v>1.3</v>
       </c>
       <c r="S6" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="T6" s="35">
         <v>5180</v>
       </c>
       <c r="U6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="V6" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="Y6" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="Z6" s="35">
         <v>780</v>
@@ -9879,16 +10081,16 @@
         <v>1.06</v>
       </c>
       <c r="AD6" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="AE6" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AF6" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="AH6" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="AI6" s="35">
         <v>-40</v>
@@ -9912,19 +10114,19 @@
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F7" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="G7" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="H7" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="J7" s="35">
         <v>6.3</v>
@@ -9936,7 +10138,7 @@
         <v>30</v>
       </c>
       <c r="M7" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="N7" s="35">
         <v>6.3</v>
@@ -9951,19 +10153,19 @@
         <v>1.3</v>
       </c>
       <c r="S7" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="T7" s="35">
         <v>5180</v>
       </c>
       <c r="U7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="V7" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="Y7" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="Z7" s="35">
         <v>630</v>
@@ -9975,16 +10177,16 @@
         <v>1.06</v>
       </c>
       <c r="AD7" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="AE7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AF7" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="AH7" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="AI7" s="35">
         <v>30</v>
@@ -10017,16 +10219,16 @@
         <v>90</v>
       </c>
       <c r="F8" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="G8" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="H8" t="s">
-        <v>210</v>
+        <v>91</v>
       </c>
       <c r="I8" t="s">
-        <v>211</v>
+        <v>92</v>
       </c>
       <c r="J8" s="35">
         <v>5.8</v>
@@ -10038,7 +10240,7 @@
         <v>20</v>
       </c>
       <c r="M8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="N8" s="35">
         <v>5.8</v>
@@ -10053,19 +10255,19 @@
         <v>1.3</v>
       </c>
       <c r="S8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="T8" s="35">
         <v>4970</v>
       </c>
       <c r="U8" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="V8" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="Y8" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="Z8" s="35">
         <v>580</v>
@@ -10077,16 +10279,16 @@
         <v>1.06</v>
       </c>
       <c r="AD8" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AE8" t="s">
         <v>90</v>
       </c>
       <c r="AF8" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="AH8" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="AI8" s="35">
         <v>20</v>
@@ -10104,7 +10306,7 @@
     </row>
     <row r="9" spans="1:42" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B9" t="s">
         <v>21</v>
@@ -10113,16 +10315,16 @@
         <v>13</v>
       </c>
       <c r="D9" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E9" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F9" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G9" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J9" s="35">
         <v>71.95</v>
@@ -10141,13 +10343,13 @@
         <v>0</v>
       </c>
       <c r="U9" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="V9" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="Y9" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="Z9" s="35">
         <v>935.35</v>
@@ -10157,19 +10359,19 @@
       </c>
       <c r="AB9" s="35"/>
       <c r="AD9" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="AE9" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="AF9" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="AG9">
         <v>13</v>
       </c>
       <c r="AH9" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="AI9" s="35"/>
       <c r="AJ9">
@@ -10179,25 +10381,25 @@
     </row>
     <row r="10" spans="1:42" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B10" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C10">
         <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E10" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F10" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="G10" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J10" s="35">
         <v>17.629899999999999</v>
@@ -10216,13 +10418,13 @@
         <v>0</v>
       </c>
       <c r="U10" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="V10" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="Y10" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="Z10" s="35">
         <v>387.86</v>
@@ -10232,19 +10434,19 @@
       </c>
       <c r="AB10" s="35"/>
       <c r="AD10" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="AE10" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AF10" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="AG10">
         <v>22</v>
       </c>
       <c r="AH10" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="AI10" s="35"/>
       <c r="AJ10">

</xml_diff>